<commit_message>
Add classification analysis script and GUIs
Add a new analyse_classifications.py tool that reads raw Zooniverse export CSVs and builds a formatted multi-sheet Excel report (overview, workflow, subject, user, answer breakdown, source image, time stats). Update README to document the new script and add openpyxl to installation instructions. Refactor export_classifications.py and import_subjects.py to use Tkinter GUI forms for interactive input, improve env file discovery/loading and authentication robustness (retries and clearer errors), and fix CSV handling (read export bytes via BytesIO). Also update tracker.xlsx. These changes improve usability for non-CLI users and provide a reusable analysis/reporting workflow.
</commit_message>
<xml_diff>
--- a/zooniverse-project/tracker.xlsx
+++ b/zooniverse-project/tracker.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="85" documentId="11_EA5DE2B7583E395B7779DB9E9EBEE0E8D6C668C3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{193547D9-1136-4937-8539-B64C0020E0E8}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="426" yWindow="426" windowWidth="20724" windowHeight="12228" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subject Set Tracker" sheetId="1" r:id="rId1"/>
@@ -2942,7 +2942,7 @@
     <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.55000000000000004">
       <c r="D4" s="40">
         <f ca="1">TODAY()</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="E4" s="35"/>
     </row>

</xml_diff>

<commit_message>
Remove personal configs & add path localization
Purge machine-specific config/log files and make toolbox image paths robust across users. Deleted per-user JSON configs and runtime logs from zooniverse-project/scripts and project root; added .gitignore entries to ignore personal Claude settings, GUI caches, generated reports and caches. Added requirements.txt and updated README to install from it. In toolbox_to_subjects.py imported re/getpass and added localize_path() to rewrite Windows user-profile paths to the current user, and applied it when checking and loading source images to avoid missing-file issues due to hardcoded usernames.
</commit_message>
<xml_diff>
--- a/zooniverse-project/tracker.xlsx
+++ b/zooniverse-project/tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thomsonr\Seattle Aquarium Dropbox\Coastal_Climate_Resilience\GitHub\CCR_benthic_analyses\zooniverse-project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://seattleaquarium-my.sharepoint.com/personal/m_williams_seattleaquarium_org/Documents/Documents/GitHub/CCR_benthic_analyses/zooniverse-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A69BFA-930D-43CD-89E2-05D4DD25F784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="13_ncr:1_{31A69BFA-930D-43CD-89E2-05D4DD25F784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62B0F3C7-5280-44AD-8495-BFDE1A5266A2}"/>
   <bookViews>
-    <workbookView xWindow="51720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subject Set Tracker" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="87">
   <si>
     <t>Track transects, subject sets, image counts, upload status &amp; script versions</t>
   </si>
@@ -261,6 +261,42 @@
   </si>
   <si>
     <t>Elliott Bay / Pocket Beach</t>
+  </si>
+  <si>
+    <t>CNL_S24_T1</t>
+  </si>
+  <si>
+    <t>CNL_S24_T2</t>
+  </si>
+  <si>
+    <t>CNL_S24_T3</t>
+  </si>
+  <si>
+    <t>CNL_S24_T4</t>
+  </si>
+  <si>
+    <t>CNL_S24_T5</t>
+  </si>
+  <si>
+    <t>CNL_S24_T6</t>
+  </si>
+  <si>
+    <t>EBM_S24_T1</t>
+  </si>
+  <si>
+    <t>EBM_S24_T2</t>
+  </si>
+  <si>
+    <t>EBM_S24_T3</t>
+  </si>
+  <si>
+    <t>EBM_S24_T4</t>
+  </si>
+  <si>
+    <t>EBM_S24_T6</t>
+  </si>
+  <si>
+    <t>Not done in Zooniverse</t>
   </si>
 </sst>
 </file>
@@ -355,7 +391,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -415,6 +451,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5F5E3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -511,7 +553,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -624,6 +666,34 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -643,32 +713,21 @@
     <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -676,6 +735,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFD5F5E3"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -972,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -988,36 +1052,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="56" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
     </row>
     <row r="2" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
     </row>
     <row r="3" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
@@ -1057,997 +1121,1278 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:12" s="64" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="61" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="63">
+        <v>45573</v>
+      </c>
+      <c r="D4" s="62"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="62" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" s="44" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="33">
+        <v>45573</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" s="64" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="61" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="63">
+        <v>45573</v>
+      </c>
+      <c r="D6" s="62"/>
+      <c r="E6" s="61"/>
+      <c r="F6" s="61"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="63"/>
+      <c r="I6" s="61"/>
+      <c r="J6" s="61"/>
+      <c r="K6" s="65"/>
+      <c r="L6" s="62" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" s="44" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="33">
+        <v>45573</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="65"/>
+      <c r="L7" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" s="64" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="61" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="63">
+        <v>45573</v>
+      </c>
+      <c r="D8" s="62"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="63"/>
+      <c r="I8" s="61"/>
+      <c r="J8" s="61"/>
+      <c r="K8" s="65"/>
+      <c r="L8" s="62" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" s="44" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="33">
+        <v>45573</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="65"/>
+      <c r="L9" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" s="64" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="63">
+        <v>45574</v>
+      </c>
+      <c r="D10" s="62"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="61"/>
+      <c r="J10" s="61"/>
+      <c r="K10" s="65"/>
+      <c r="L10" s="62" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" s="44" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="33">
+        <f>$C$10</f>
+        <v>45574</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="65"/>
+      <c r="L11" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" s="64" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="63">
+        <v>45574</v>
+      </c>
+      <c r="D12" s="62"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="65"/>
+      <c r="L12" s="62" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" s="44" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="33">
+        <f>$C$10</f>
+        <v>45574</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="65"/>
+      <c r="L13" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" s="64" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="63">
+        <v>45574</v>
+      </c>
+      <c r="D14" s="62"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="63"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="65"/>
+      <c r="L14" s="62" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" s="44" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="33">
+        <f>$C$10</f>
+        <v>45574</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="65"/>
+      <c r="L15" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" s="64" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="61"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="63"/>
+      <c r="D16" s="62"/>
+      <c r="E16" s="61"/>
+      <c r="F16" s="61"/>
+      <c r="G16" s="61"/>
+      <c r="H16" s="63"/>
+      <c r="I16" s="61"/>
+      <c r="J16" s="61"/>
+      <c r="K16" s="61"/>
+      <c r="L16" s="62"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="33">
+      <c r="C17" s="33">
         <v>45684</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E17" s="2">
         <v>135009</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F17" s="2">
         <v>66</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G17" s="2">
         <v>3100</v>
       </c>
-      <c r="H4" s="33">
+      <c r="H17" s="33">
         <v>46105</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="6" t="s">
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="34">
+        <v>45684</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="4">
+        <v>135018</v>
+      </c>
+      <c r="F18" s="4">
+        <v>71</v>
+      </c>
+      <c r="G18" s="4">
+        <v>3350</v>
+      </c>
+      <c r="H18" s="34">
+        <v>46105</v>
+      </c>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="33">
+        <v>45685</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E19" s="2">
+        <v>135048</v>
+      </c>
+      <c r="F19" s="2">
+        <v>64</v>
+      </c>
+      <c r="G19" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H19" s="33">
+        <v>46105</v>
+      </c>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="34">
+        <v>45685</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="4">
+        <v>135054</v>
+      </c>
+      <c r="F20" s="4">
+        <v>62</v>
+      </c>
+      <c r="G20" s="4">
+        <v>2900</v>
+      </c>
+      <c r="H20" s="34">
+        <v>46105</v>
+      </c>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="33">
+        <v>45684</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="2">
+        <v>135378</v>
+      </c>
+      <c r="F21" s="2">
+        <v>66</v>
+      </c>
+      <c r="G21" s="2">
+        <v>3300</v>
+      </c>
+      <c r="H21" s="33">
+        <v>46117</v>
+      </c>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="34">
+        <v>45685</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E22" s="4">
+        <v>135306</v>
+      </c>
+      <c r="F22" s="4">
+        <v>56</v>
+      </c>
+      <c r="G22" s="4">
+        <v>2800</v>
+      </c>
+      <c r="H22" s="34">
+        <v>46115</v>
+      </c>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="33">
+        <v>45684</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="2">
+        <v>135393</v>
+      </c>
+      <c r="F23" s="2">
+        <v>60</v>
+      </c>
+      <c r="G23" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H23" s="33">
+        <v>46118</v>
+      </c>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="34">
+        <v>45685</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" s="4">
+        <v>135399</v>
+      </c>
+      <c r="F24" s="4">
+        <v>60</v>
+      </c>
+      <c r="G24" s="4">
+        <v>3000</v>
+      </c>
+      <c r="H24" s="34">
+        <v>46118</v>
+      </c>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="33">
+        <v>45684</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" s="2">
+        <v>135757</v>
+      </c>
+      <c r="F25" s="2">
+        <v>64</v>
+      </c>
+      <c r="G25" s="2">
+        <v>3200</v>
+      </c>
+      <c r="H25" s="33">
+        <v>46132</v>
+      </c>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="34">
+        <v>45685</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E26" s="4">
+        <v>135765</v>
+      </c>
+      <c r="F26" s="4">
+        <v>58</v>
+      </c>
+      <c r="G26" s="4">
+        <v>2900</v>
+      </c>
+      <c r="H26" s="34">
+        <v>46132</v>
+      </c>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="33">
+        <v>45684</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" s="2">
+        <v>135910</v>
+      </c>
+      <c r="F27" s="2">
+        <v>60</v>
+      </c>
+      <c r="G27" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H27" s="33">
+        <v>46135</v>
+      </c>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" s="43" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A28" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" s="39" t="s">
+        <v>44</v>
+      </c>
+      <c r="C28" s="40">
+        <v>45685</v>
+      </c>
+      <c r="D28" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="E28" s="38">
+        <v>135913</v>
+      </c>
+      <c r="F28" s="38">
+        <v>58</v>
+      </c>
+      <c r="G28" s="38">
+        <v>2900</v>
+      </c>
+      <c r="H28" s="40">
+        <v>46135</v>
+      </c>
+      <c r="I28" s="38"/>
+      <c r="J28" s="38"/>
+      <c r="K28" s="66" t="s">
+        <v>14</v>
+      </c>
+      <c r="L28" s="42" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="37">
+        <v>45938</v>
+      </c>
+      <c r="D29" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" s="35">
+        <v>136807</v>
+      </c>
+      <c r="F29" s="35">
+        <v>58</v>
+      </c>
+      <c r="G29" s="35">
+        <v>2800</v>
+      </c>
+      <c r="H29" s="37">
+        <v>46169</v>
+      </c>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
+      <c r="K29" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L29" s="36" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C5" s="34">
-        <v>45684</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="4">
-        <v>135018</v>
-      </c>
-      <c r="F5" s="4">
+    <row r="30" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="4">
+      <c r="B30" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="34">
+        <v>45938</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E30" s="4">
+        <v>136811</v>
+      </c>
+      <c r="F30" s="4">
+        <v>67</v>
+      </c>
+      <c r="G30" s="4">
         <v>3350</v>
       </c>
-      <c r="H5" s="34">
-        <v>46105</v>
-      </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="6" t="s">
+      <c r="H30" s="34">
+        <v>46169</v>
+      </c>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L30" s="7" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="33">
-        <v>45685</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="2">
-        <v>135048</v>
-      </c>
-      <c r="F6" s="2">
-        <v>64</v>
-      </c>
-      <c r="G6" s="2">
-        <v>3000</v>
-      </c>
-      <c r="H6" s="33">
-        <v>46105</v>
-      </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="6" t="s">
+    <row r="31" spans="1:12" s="43" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A31" s="49" t="s">
+        <v>72</v>
+      </c>
+      <c r="B31" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="51">
+        <v>45938</v>
+      </c>
+      <c r="D31" s="50" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="49">
+        <v>136817</v>
+      </c>
+      <c r="F31" s="49">
+        <v>82</v>
+      </c>
+      <c r="G31" s="49">
+        <v>4100</v>
+      </c>
+      <c r="H31" s="52">
+        <v>46169</v>
+      </c>
+      <c r="I31" s="49"/>
+      <c r="J31" s="49"/>
+      <c r="K31" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L31" s="53" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="34">
-        <v>45685</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E7" s="4">
-        <v>135054</v>
-      </c>
-      <c r="F7" s="4">
-        <v>62</v>
-      </c>
-      <c r="G7" s="4">
-        <v>2900</v>
-      </c>
-      <c r="H7" s="34">
-        <v>46105</v>
-      </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="6" t="s">
+    <row r="32" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" s="46" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="47" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32" s="48">
+        <v>45883</v>
+      </c>
+      <c r="D32" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="E32" s="46">
+        <v>137510</v>
+      </c>
+      <c r="F32" s="46">
+        <v>70</v>
+      </c>
+      <c r="G32" s="46">
+        <v>3500</v>
+      </c>
+      <c r="H32" s="48">
+        <v>46211</v>
+      </c>
+      <c r="I32" s="46"/>
+      <c r="J32" s="46"/>
+      <c r="K32" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="L32" s="47" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="33">
-        <v>45684</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E8" s="2">
-        <v>135378</v>
-      </c>
-      <c r="F8" s="2">
-        <v>66</v>
-      </c>
-      <c r="G8" s="2">
-        <v>3300</v>
-      </c>
-      <c r="H8" s="33">
-        <v>46117</v>
-      </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="34">
-        <v>45685</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E9" s="4">
-        <v>135306</v>
-      </c>
-      <c r="F9" s="4">
-        <v>56</v>
-      </c>
-      <c r="G9" s="4">
-        <v>2800</v>
-      </c>
-      <c r="H9" s="34">
-        <v>46115</v>
-      </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="33">
-        <v>45684</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" s="2">
-        <v>135393</v>
-      </c>
-      <c r="F10" s="2">
-        <v>60</v>
-      </c>
-      <c r="G10" s="2">
-        <v>3000</v>
-      </c>
-      <c r="H10" s="33">
-        <v>46118</v>
-      </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="34">
-        <v>45685</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="4">
-        <v>135399</v>
-      </c>
-      <c r="F11" s="4">
-        <v>60</v>
-      </c>
-      <c r="G11" s="4">
-        <v>3000</v>
-      </c>
-      <c r="H11" s="34">
-        <v>46118</v>
-      </c>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="33">
-        <v>45684</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" s="2">
-        <v>135757</v>
-      </c>
-      <c r="F12" s="2">
-        <v>64</v>
-      </c>
-      <c r="G12" s="2">
-        <v>3200</v>
-      </c>
-      <c r="H12" s="33">
-        <v>46132</v>
-      </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L12" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="34">
-        <v>45685</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E13" s="4">
-        <v>135765</v>
-      </c>
-      <c r="F13" s="4">
-        <v>58</v>
-      </c>
-      <c r="G13" s="4">
-        <v>2900</v>
-      </c>
-      <c r="H13" s="34">
-        <v>46132</v>
-      </c>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="33">
-        <v>45684</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E14" s="2">
-        <v>135910</v>
-      </c>
-      <c r="F14" s="2">
-        <v>60</v>
-      </c>
-      <c r="G14" s="2">
-        <v>3000</v>
-      </c>
-      <c r="H14" s="33">
-        <v>46135</v>
-      </c>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L14" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" s="43" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="40">
-        <v>45685</v>
-      </c>
-      <c r="D15" s="39" t="s">
-        <v>68</v>
-      </c>
-      <c r="E15" s="38">
-        <v>135913</v>
-      </c>
-      <c r="F15" s="38">
-        <v>58</v>
-      </c>
-      <c r="G15" s="38">
-        <v>2900</v>
-      </c>
-      <c r="H15" s="40">
-        <v>46135</v>
-      </c>
-      <c r="I15" s="38"/>
-      <c r="J15" s="38"/>
-      <c r="K15" s="41" t="s">
-        <v>16</v>
-      </c>
-      <c r="L15" s="42" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="B16" s="36" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" s="37">
-        <v>45938</v>
-      </c>
-      <c r="D16" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="35">
-        <v>136807</v>
-      </c>
-      <c r="F16" s="35">
-        <v>58</v>
-      </c>
-      <c r="G16" s="35">
-        <v>2800</v>
-      </c>
-      <c r="H16" s="37">
-        <v>46169</v>
-      </c>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L16" s="36" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B17" s="51" t="s">
-        <v>70</v>
-      </c>
-      <c r="C17" s="34">
-        <v>45938</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E17" s="4">
-        <v>136811</v>
-      </c>
-      <c r="F17" s="4">
-        <v>67</v>
-      </c>
-      <c r="G17" s="4">
-        <v>3350</v>
-      </c>
-      <c r="H17" s="34">
-        <v>46169</v>
-      </c>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L17" s="7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" s="43" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A18" s="55" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" s="56" t="s">
-        <v>70</v>
-      </c>
-      <c r="C18" s="57">
-        <v>45938</v>
-      </c>
-      <c r="D18" s="56" t="s">
-        <v>72</v>
-      </c>
-      <c r="E18" s="55">
-        <v>136817</v>
-      </c>
-      <c r="F18" s="55">
-        <v>82</v>
-      </c>
-      <c r="G18" s="55">
-        <v>4100</v>
-      </c>
-      <c r="H18" s="58">
-        <v>46169</v>
-      </c>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="41" t="s">
-        <v>16</v>
-      </c>
-      <c r="L18" s="59" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="52" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="53" t="s">
-        <v>74</v>
-      </c>
-      <c r="C19" s="54">
-        <v>45883</v>
-      </c>
-      <c r="D19" s="53" t="s">
-        <v>73</v>
-      </c>
-      <c r="E19" s="52">
-        <v>137510</v>
-      </c>
-      <c r="F19" s="52">
-        <v>70</v>
-      </c>
-      <c r="G19" s="52">
-        <v>3500</v>
-      </c>
-      <c r="H19" s="54">
-        <v>46211</v>
-      </c>
-      <c r="I19" s="52"/>
-      <c r="J19" s="52"/>
-      <c r="K19" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="L19" s="53" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="2"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="33"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="33"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="8"/>
-    </row>
-    <row r="21" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="4"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="7"/>
-    </row>
-    <row r="22" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="2"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="8"/>
-    </row>
-    <row r="23" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="4"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="7"/>
-    </row>
-    <row r="24" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="2"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="8"/>
-    </row>
-    <row r="25" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="4"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="7"/>
-    </row>
-    <row r="26" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="2"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="33"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="8"/>
-    </row>
-    <row r="27" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="4"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="34"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="7"/>
-    </row>
-    <row r="28" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="2"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="8"/>
-    </row>
-    <row r="29" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="4"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="7"/>
-    </row>
-    <row r="30" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="2"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="33"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="33"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="8"/>
-    </row>
-    <row r="31" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="4"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="7"/>
-    </row>
-    <row r="32" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="2"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="33"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="8"/>
-    </row>
     <row r="33" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="4"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="7"/>
+      <c r="A33" s="2"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="33"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+      <c r="L33" s="8"/>
     </row>
     <row r="34" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="2"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="33"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="8"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="34"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="7"/>
     </row>
     <row r="35" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="4"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="7"/>
+      <c r="A35" s="2"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="8"/>
     </row>
     <row r="36" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="2"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="33"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="8"/>
+      <c r="A36" s="4"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="34"/>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="7"/>
     </row>
     <row r="37" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="4"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="34"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="7"/>
+      <c r="A37" s="2"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="33"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="8"/>
     </row>
     <row r="38" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="2"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="33"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="8"/>
+      <c r="A38" s="4"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="34"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="7"/>
     </row>
     <row r="39" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="4"/>
-      <c r="B39" s="7"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4"/>
-      <c r="L39" s="7"/>
+      <c r="A39" s="2"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+      <c r="L39" s="8"/>
     </row>
     <row r="40" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="2"/>
-      <c r="B40" s="8"/>
-      <c r="C40" s="33"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="8"/>
+      <c r="A40" s="4"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="34"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="7"/>
     </row>
     <row r="41" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="4"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="34"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="7"/>
+      <c r="A41" s="2"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="33"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+      <c r="L41" s="8"/>
     </row>
     <row r="42" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="2"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="33"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
-      <c r="L42" s="8"/>
+      <c r="A42" s="4"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="34"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="34"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="7"/>
     </row>
     <row r="43" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" s="4"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4"/>
-      <c r="L43" s="7"/>
+      <c r="A43" s="2"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="33"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+      <c r="L43" s="8"/>
     </row>
     <row r="44" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="2"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="33"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
-      <c r="L44" s="8"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="34"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="34"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="7"/>
     </row>
     <row r="45" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" s="4"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="34"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="7"/>
+      <c r="A45" s="2"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+      <c r="L45" s="8"/>
     </row>
     <row r="46" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="2"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-      <c r="L46" s="8"/>
+      <c r="A46" s="4"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="7"/>
     </row>
     <row r="47" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="4"/>
-      <c r="B47" s="7"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="4"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="7"/>
+      <c r="A47" s="2"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+      <c r="L47" s="8"/>
     </row>
     <row r="48" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="2"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2"/>
-      <c r="H48" s="2"/>
-      <c r="I48" s="2"/>
-      <c r="J48" s="2"/>
-      <c r="K48" s="2"/>
-      <c r="L48" s="8"/>
+      <c r="A48" s="4"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="34"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="7"/>
     </row>
     <row r="49" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" s="4"/>
-      <c r="B49" s="7"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="7"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
-      <c r="J49" s="4"/>
-      <c r="K49" s="4"/>
-      <c r="L49" s="7"/>
+      <c r="A49" s="2"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+      <c r="J49" s="2"/>
+      <c r="K49" s="2"/>
+      <c r="L49" s="8"/>
     </row>
     <row r="50" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A50" s="2"/>
-      <c r="B50" s="8"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="2"/>
-      <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
-      <c r="L50" s="8"/>
+      <c r="A50" s="4"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="34"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="7"/>
     </row>
     <row r="51" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A51" s="4"/>
-      <c r="B51" s="7"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-      <c r="K51" s="4"/>
-      <c r="L51" s="7"/>
+      <c r="A51" s="2"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="33"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
+      <c r="L51" s="8"/>
+    </row>
+    <row r="52" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A52" s="4"/>
+      <c r="B52" s="7"/>
+      <c r="C52" s="34"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+      <c r="L52" s="7"/>
+    </row>
+    <row r="53" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A53" s="2"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="33"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
+      <c r="L53" s="8"/>
+    </row>
+    <row r="54" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" s="4"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="34"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+      <c r="L54" s="7"/>
+    </row>
+    <row r="55" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A55" s="2"/>
+      <c r="B55" s="8"/>
+      <c r="C55" s="33"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="2"/>
+      <c r="L55" s="8"/>
+    </row>
+    <row r="56" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A56" s="4"/>
+      <c r="B56" s="7"/>
+      <c r="C56" s="34"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+      <c r="H56" s="4"/>
+      <c r="I56" s="4"/>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4"/>
+      <c r="L56" s="7"/>
+    </row>
+    <row r="57" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A57" s="2"/>
+      <c r="B57" s="8"/>
+      <c r="C57" s="33"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+      <c r="K57" s="2"/>
+      <c r="L57" s="8"/>
+    </row>
+    <row r="58" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A58" s="4"/>
+      <c r="B58" s="7"/>
+      <c r="C58" s="34"/>
+      <c r="D58" s="7"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+      <c r="K58" s="4"/>
+      <c r="L58" s="7"/>
+    </row>
+    <row r="59" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A59" s="2"/>
+      <c r="B59" s="8"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
+      <c r="L59" s="8"/>
+    </row>
+    <row r="60" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A60" s="4"/>
+      <c r="B60" s="7"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="7"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="I60" s="4"/>
+      <c r="J60" s="4"/>
+      <c r="K60" s="4"/>
+      <c r="L60" s="7"/>
+    </row>
+    <row r="61" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A61" s="2"/>
+      <c r="B61" s="8"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="8"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
+      <c r="L61" s="8"/>
+    </row>
+    <row r="62" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A62" s="4"/>
+      <c r="B62" s="7"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+      <c r="L62" s="7"/>
+    </row>
+    <row r="63" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A63" s="2"/>
+      <c r="B63" s="8"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="8"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
+      <c r="I63" s="2"/>
+      <c r="J63" s="2"/>
+      <c r="K63" s="2"/>
+      <c r="L63" s="8"/>
+    </row>
+    <row r="64" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A64" s="4"/>
+      <c r="B64" s="7"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+      <c r="L64" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2056,7 +2401,7 @@
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="K4:K198" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="K4:K211" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Uploaded,Uploaded,In Progress,Awaiting Export,Complete,On Hold"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2078,32 +2423,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
     </row>
     <row r="2" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="10" t="s">
@@ -2730,40 +3075,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
     </row>
     <row r="3" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="13" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="14">
-        <f>COUNTA('Subject Set Tracker'!A4:A198)</f>
-        <v>16</v>
-      </c>
-      <c r="D3" s="48" t="s">
+        <f>COUNTA('Subject Set Tracker'!A5:A211)</f>
+        <v>27</v>
+      </c>
+      <c r="D3" s="58" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="45"/>
+      <c r="E3" s="55"/>
     </row>
     <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.55000000000000004">
-      <c r="D4" s="50">
+      <c r="D4" s="60">
         <f ca="1">TODAY()</f>
-        <v>46212</v>
-      </c>
-      <c r="E4" s="45"/>
+        <v>46217</v>
+      </c>
+      <c r="E4" s="55"/>
     </row>
     <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="13" t="s">
         <v>35</v>
       </c>
       <c r="B5" s="14">
-        <f>SUM('Subject Set Tracker'!F4:F198)</f>
+        <f>SUM('Subject Set Tracker'!F5:F211)</f>
         <v>1022</v>
       </c>
     </row>
@@ -2778,7 +3123,7 @@
         <v>37</v>
       </c>
       <c r="B7" s="14">
-        <f>SUM('Subject Set Tracker'!G4:G198)</f>
+        <f>SUM('Subject Set Tracker'!G5:G211)</f>
         <v>50200</v>
       </c>
       <c r="D7" s="17" t="s">
@@ -2797,8 +3142,8 @@
         <v>14</v>
       </c>
       <c r="B9" s="22">
-        <f>COUNTIF('Subject Set Tracker'!K4:K198,"Complete")</f>
-        <v>0</v>
+        <f>COUNTIF('Subject Set Tracker'!K5:K211,"Complete")</f>
+        <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
         <v>15</v>
@@ -2816,8 +3161,8 @@
         <v>16</v>
       </c>
       <c r="B11" s="14">
-        <f>COUNTIF('Subject Set Tracker'!K4:K198,"In Progress")</f>
-        <v>16</v>
+        <f>COUNTIF('Subject Set Tracker'!K5:K211,"In Progress")</f>
+        <v>4</v>
       </c>
       <c r="D11" s="27" t="s">
         <v>38</v>
@@ -2829,7 +3174,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="30">
-        <f>COUNTIF('Subject Set Tracker'!K4:K198,"Awaiting Export")</f>
+        <f>COUNTIF('Subject Set Tracker'!K5:K211,"Awaiting Export")</f>
         <v>0</v>
       </c>
     </row>
@@ -2838,7 +3183,7 @@
         <v>17</v>
       </c>
       <c r="B15" s="32">
-        <f>COUNTIF('Subject Set Tracker'!K4:K198,"Not Uploaded")</f>
+        <f>COUNTIF('Subject Set Tracker'!K5:K211,"Not Uploaded")</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>